<commit_message>
vault backup: 2024-03-12 09:43:30
</commit_message>
<xml_diff>
--- a/public/assets/excel_router_task.xlsx
+++ b/public/assets/excel_router_task.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcc\git\informatikgarten.ch\content\3 Computer &amp; Netzwerke\2 Netzwerke und das Internet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcc\git\informatikgarten.ch\content\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B126203D-2C40-41EB-B497-839DCC330E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431794FB-B180-49BC-8C91-7CBA24624346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" activeTab="2" xr2:uid="{8B4C5CB2-983E-4FDC-89E4-8A1111F2665D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" activeTab="1" xr2:uid="{8B4C5CB2-983E-4FDC-89E4-8A1111F2665D}"/>
   </bookViews>
   <sheets>
     <sheet name="Einstieg" sheetId="1" r:id="rId1"/>
-    <sheet name="Binäre Erklärung" sheetId="3" r:id="rId2"/>
+    <sheet name="Binäre Erklärung" sheetId="4" r:id="rId2"/>
     <sheet name="IP-Router" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="98">
   <si>
     <t>Einstieg: Excel-Formeln</t>
   </si>
@@ -279,9 +279,6 @@
     <t>Dezimal</t>
   </si>
   <si>
-    <t>Netzwerk-Adr.</t>
-  </si>
-  <si>
     <t>101</t>
   </si>
   <si>
@@ -424,12 +421,126 @@
   <si>
     <t>Bitweise Vergleichen mit "bitand" / "bitund"</t>
   </si>
+  <si>
+    <r>
+      <t>Grundidee: Wir schauen, ob durch ein Bitwise AND (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) mit der gleichen Subnetmaske nochmal die gleiche Netzwerkadresse entsteht. Falls ja, ist es das gleiche Netzwerk!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>👆</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> daraus ergibt sich folgende Netzwerkadresse:</t>
+    </r>
+  </si>
+  <si>
+    <t>Byte</t>
+  </si>
+  <si>
+    <t>Meine IP</t>
+  </si>
+  <si>
+    <t>Netzwerk-Adresse (tiefste Adresse)</t>
+  </si>
+  <si>
+    <t>1. IP für Gerät (oft der Gateway)</t>
+  </si>
+  <si>
+    <t>2. IP für Gerät (oft der Gateway)</t>
+  </si>
+  <si>
+    <t>…alle weiteren IPs die Geräte…</t>
+  </si>
+  <si>
+    <t>Letzte IP für Gerät</t>
+  </si>
+  <si>
+    <t>Broadcast-Adresse (höchste Adresse)</t>
+  </si>
+  <si>
+    <t>👆 daraus kann man das gesamte Netzwerk herleiten:</t>
+  </si>
+  <si>
+    <t>Welche IP-Adressen gehören also zum gleichen Netzwerk?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Die Subnetmaske zieht also </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>eine</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> klare Grenze.</t>
+    </r>
+  </si>
+  <si>
+    <t>Sie muss deswegen aus einer Serie '1' sein und dann nur noch '0'.</t>
+  </si>
+  <si>
+    <t>Subnetmasken mit mehr als einer Grenze zwischen '1' zu '0' sind ungültig!</t>
+  </si>
+  <si>
+    <t>Die einzigen möglichen Dezimalzahlen sind:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -495,8 +606,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -578,6 +721,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFAFAF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -763,7 +912,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -791,38 +940,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -832,27 +980,45 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -880,56 +1046,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1186,23 +1302,26 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>545171</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>120001</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>99837</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>178739</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>725000</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>39175</xdr:rowOff>
+      <xdr:colOff>602075</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Rectangle 1">
+        <xdr:cNvPr id="3" name="Oval 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29A35466-7298-4D64-A1C3-E7993A30D238}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E19F3B53-143E-4FF2-A3A1-63B71EDF6B40}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{29A35466-7298-4D64-A1C3-E7993A30D238}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1210,27 +1329,23 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4545171" y="685001"/>
-          <a:ext cx="2449829" cy="1629174"/>
+          <a:off x="7510287" y="2267889"/>
+          <a:ext cx="603838" cy="202261"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FF0000">
-            <a:alpha val="9020"/>
-          </a:srgbClr>
-        </a:solidFill>
-        <a:ln>
+        <a:noFill/>
+        <a:ln w="38100">
           <a:solidFill>
-            <a:srgbClr val="C00000"/>
+            <a:srgbClr val="FF0000"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
           <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
+            <a:shade val="15000"/>
           </a:schemeClr>
         </a:lnRef>
         <a:fillRef idx="1">
@@ -1248,7 +1363,987 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="l"/>
-          <a:endParaRPr lang="de-CH" sz="1100"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>587964</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>183444</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>65855</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>70791</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA3CFB93-F78A-417C-8DCA-2D518AC08BAC}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3E62796F-241B-F541-067D-137D3746E82A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5814014" y="1891594"/>
+          <a:ext cx="824091" cy="268347"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>530413</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>173868</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>698510</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>75595</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="10" name="Gruppieren 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26D939B1-D605-7D14-B7C1-3E3B3EEB3025}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="5754044" y="362856"/>
+          <a:ext cx="2443514" cy="5465537"/>
+          <a:chOff x="5754044" y="362856"/>
+          <a:chExt cx="2443514" cy="5397501"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="Rectangle 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61587E41-A932-40B5-887E-2CC6F531D394}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5835952" y="362856"/>
+            <a:ext cx="2281128" cy="5397501"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FF0000">
+              <a:alpha val="9020"/>
+            </a:srgbClr>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="de-CH" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="5" name="Textfeld 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5270A598-FC4F-435F-A0E7-66171F2D3C55}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5754044" y="778631"/>
+            <a:ext cx="2443514" cy="596047"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="2000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Netzwerkteil</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>(definiert durch Subnetmaske)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>18814</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>28222</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>296331</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>11524</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A359104-CCF1-4E63-B294-B63ED97DD786}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3E62796F-241B-F541-067D-137D3746E82A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3016014" y="1926872"/>
+          <a:ext cx="277517" cy="173802"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>111949</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>23518</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>4704</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>183445</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D125D9A1-0C32-4483-B525-EEBC6A154AD1}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3E62796F-241B-F541-067D-137D3746E82A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3864799" y="2303168"/>
+          <a:ext cx="337255" cy="159927"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>323894</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>23359</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>663302</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>183286</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E1962ED-D877-4FDF-93FD-D90F5120385A}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3E62796F-241B-F541-067D-137D3746E82A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7835944" y="1541009"/>
+          <a:ext cx="339408" cy="159927"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>97877</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>17979</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>308132</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>177906</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8739814-F73C-4A54-B586-1CBA6670E473}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3E62796F-241B-F541-067D-137D3746E82A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3850727" y="1535629"/>
+          <a:ext cx="337255" cy="159927"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -1261,16 +2356,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>41412</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>165651</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>160474</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>76355</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>175351</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>615156</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>86055</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1300,8 +2395,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="3975651" y="2767771"/>
-          <a:ext cx="4693479" cy="1127852"/>
+          <a:off x="7145474" y="6733933"/>
+          <a:ext cx="4691323" cy="1140794"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1322,16 +2417,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>351368</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>155721</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>490274</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>66425</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>12050</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>155721</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>150956</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>66425</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1346,8 +2441,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="6924680" y="4049499"/>
-          <a:ext cx="1093033" cy="269657"/>
+          <a:off x="10068857" y="8099170"/>
+          <a:ext cx="1131094" cy="265916"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1400,16 +2495,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>18467</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>154008</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>157373</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>64712</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>288124</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>154009</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>427030</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>64713</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1424,8 +2519,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="6591779" y="4047786"/>
-          <a:ext cx="1093034" cy="269657"/>
+          <a:off x="9737826" y="8095587"/>
+          <a:ext cx="1131095" cy="269657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1478,16 +2573,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>411188</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140535</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>351657</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>51239</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>71869</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>140536</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>12337</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>51240</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1502,8 +2597,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="5579172" y="4034313"/>
-          <a:ext cx="1093034" cy="269657"/>
+          <a:off x="8719770" y="8083985"/>
+          <a:ext cx="1131095" cy="265915"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1553,9 +2648,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1593,7 +2688,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1699,7 +2794,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1841,7 +2936,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2493,7 +3588,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
@@ -2512,7 +3607,7 @@
         <v>5</v>
       </c>
       <c r="C95" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E95">
         <v>5</v>
@@ -2576,12 +3671,12 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
@@ -2626,7 +3721,7 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
@@ -2634,12 +3729,12 @@
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
@@ -2776,17 +3871,17 @@
     </row>
     <row r="137" spans="1:10" s="9" customFormat="1" ht="31" x14ac:dyDescent="0.7">
       <c r="A137" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
@@ -2839,27 +3934,27 @@
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A151" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B151">
         <v>1</v>
@@ -2894,12 +3989,12 @@
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A157" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B157">
         <v>1</v>
@@ -3019,661 +4114,1308 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC0886E-6230-44AA-AB02-85890F3B0BBF}">
-  <dimension ref="A2:T16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A06155BC-C582-4FCE-8043-D04D3A7FCBBD}">
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="1.7265625" customWidth="1"/>
-    <col min="4" max="4" width="5.08984375" customWidth="1"/>
-    <col min="5" max="5" width="1.81640625" customWidth="1"/>
-    <col min="6" max="6" width="5.54296875" customWidth="1"/>
-    <col min="7" max="7" width="1.453125" customWidth="1"/>
-    <col min="8" max="8" width="5.90625" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="1.453125" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="1.453125" customWidth="1"/>
-    <col min="15" max="15" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="1.453125" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.90625" customWidth="1"/>
+    <col min="2" max="2" width="4.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="1.7265625" style="20" customWidth="1"/>
+    <col min="4" max="4" width="4.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="1.81640625" style="20" customWidth="1"/>
+    <col min="6" max="6" width="4.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="1.453125" style="20" customWidth="1"/>
+    <col min="8" max="8" width="4.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="1.453125" style="20" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="1.453125" style="20" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="1.453125" style="20" customWidth="1"/>
+    <col min="17" max="17" width="10.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.1796875" customWidth="1"/>
-    <col min="21" max="21" width="10.6328125" customWidth="1"/>
+    <col min="21" max="21" width="10.54296875" customWidth="1"/>
     <col min="22" max="22" width="10.26953125" customWidth="1"/>
+    <col min="23" max="23" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="S2" s="14" t="s">
+    <row r="1" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="T1" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="U1" s="11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="S3" s="16">
+      <c r="W1" s="11"/>
+    </row>
+    <row r="2" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A2" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="54">
+        <v>1</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54">
+        <v>2</v>
+      </c>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54">
+        <v>3</v>
+      </c>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54">
+        <v>4</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="54">
+        <v>1</v>
+      </c>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54">
+        <v>2</v>
+      </c>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54">
+        <v>3</v>
+      </c>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A3" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="60">
+        <v>192</v>
+      </c>
+      <c r="C3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="60">
+        <v>168</v>
+      </c>
+      <c r="E3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="60">
+        <v>6</v>
+      </c>
+      <c r="G3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="60">
+        <v>6</v>
+      </c>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="60" t="str">
+        <f>DEC2BIN(B3,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="60" t="str">
+        <f>DEC2BIN(D3,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="60" t="str">
+        <f>DEC2BIN(F3,8)</f>
+        <v>00000110</v>
+      </c>
+      <c r="P3" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q3" s="60" t="str">
+        <f>DEC2BIN(H3,8)</f>
+        <v>00000110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A4" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="60">
         <v>255</v>
       </c>
-      <c r="T3" s="11" t="str">
-        <f>DEC2BIN(S3,8)</f>
+      <c r="C4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="60">
+        <v>255</v>
+      </c>
+      <c r="E4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="60">
+        <v>254</v>
+      </c>
+      <c r="G4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="60">
+        <v>0</v>
+      </c>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="60" t="str">
+        <f>DEC2BIN(B4,8)</f>
         <v>11111111</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="S4" s="11">
-        <v>254</v>
-      </c>
-      <c r="T4" s="11" t="str">
-        <f t="shared" ref="T4:T11" si="0">DEC2BIN(S4,8)</f>
+      <c r="L4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="60" t="str">
+        <f>DEC2BIN(D4,8)</f>
+        <v>11111111</v>
+      </c>
+      <c r="N4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="60" t="str">
+        <f>DEC2BIN(F4,8)</f>
         <v>11111110</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="A5" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="12">
+      <c r="P4" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q4" s="60" t="str">
+        <f>DEC2BIN(H4,8)</f>
+        <v>00000000</v>
+      </c>
+      <c r="W4" s="11"/>
+    </row>
+    <row r="5" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="S5" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="V5" s="11"/>
+    </row>
+    <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="S6" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="V6" s="11"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="S7" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A8" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="V8" s="11"/>
+    </row>
+    <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A9" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="62">
+        <f>_xlfn.BITAND($B$3,$B$4)</f>
         <v>192</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="12">
+      <c r="C9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="62">
+        <f>_xlfn.BITAND($D$3,$D$4)</f>
         <v>168</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="12">
-        <v>2</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="12">
-        <v>13</v>
-      </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="12" t="str">
-        <f t="shared" ref="K5:K10" si="1">DEC2BIN(B5,8)</f>
-        <v>11000000</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M5" s="12" t="str">
-        <f t="shared" ref="M5:M10" si="2">DEC2BIN(D5,8)</f>
-        <v>10101000</v>
-      </c>
-      <c r="N5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O5" s="12" t="str">
-        <f t="shared" ref="O5:O10" si="3">DEC2BIN(F5,8)</f>
-        <v>00000010</v>
-      </c>
-      <c r="P5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q5" s="12" t="str">
-        <f t="shared" ref="Q5:Q10" si="4">DEC2BIN(H5,8)</f>
-        <v>00001101</v>
-      </c>
-      <c r="S5" s="16">
-        <v>252</v>
-      </c>
-      <c r="T5" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>11111100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="A6" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="12">
-        <v>192</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="12">
-        <v>168</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" s="12">
-        <v>2</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="12">
-        <v>41</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="12" t="str">
-        <f t="shared" si="1"/>
-        <v>11000000</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" s="12" t="str">
-        <f t="shared" si="2"/>
-        <v>10101000</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O6" s="12" t="str">
-        <f t="shared" si="3"/>
-        <v>00000010</v>
-      </c>
-      <c r="P6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q6" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>00101001</v>
-      </c>
-      <c r="S6" s="11">
-        <v>248</v>
-      </c>
-      <c r="T6" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>11111000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="A7" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="12">
-        <v>192</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="12">
-        <v>168</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="12">
-        <v>2</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="12">
-        <v>51</v>
-      </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" s="12" t="str">
-        <f t="shared" si="1"/>
-        <v>11000000</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M7" s="12" t="str">
-        <f t="shared" si="2"/>
-        <v>10101000</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O7" s="12" t="str">
-        <f t="shared" si="3"/>
-        <v>00000010</v>
-      </c>
-      <c r="P7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q7" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>00110011</v>
-      </c>
-      <c r="S7" s="11">
-        <v>240</v>
-      </c>
-      <c r="T7" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>11110000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="A8" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="12">
-        <v>192</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="12">
-        <v>168</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="12">
-        <v>2</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="12">
-        <v>23</v>
-      </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K8" s="12" t="str">
-        <f t="shared" si="1"/>
-        <v>11000000</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M8" s="12" t="str">
-        <f t="shared" si="2"/>
-        <v>10101000</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O8" s="12" t="str">
-        <f t="shared" si="3"/>
-        <v>00000010</v>
-      </c>
-      <c r="P8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q8" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>00010111</v>
-      </c>
-      <c r="S8" s="11">
-        <v>224</v>
-      </c>
-      <c r="T8" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>11100000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
-      <c r="A9" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="12">
-        <v>192</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="12">
-        <v>168</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="12">
-        <v>2</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="12">
-        <v>23</v>
+      <c r="E9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="62">
+        <f>_xlfn.BITAND($F$3,$F$4)</f>
+        <v>6</v>
+      </c>
+      <c r="G9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="62">
+        <f>_xlfn.BITAND($H$3,$H$4)</f>
+        <v>0</v>
       </c>
       <c r="I9" s="12"/>
       <c r="J9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="12" t="str">
+      <c r="K9" s="62" t="str">
+        <f>DEC2BIN(B9,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" s="62" t="str">
+        <f t="shared" ref="M9:Q9" si="0">DEC2BIN(D9,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="O9" s="62" t="str">
+        <f t="shared" si="0"/>
+        <v>00000110</v>
+      </c>
+      <c r="P9" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q9" s="62" t="str">
+        <f t="shared" si="0"/>
+        <v>00000000</v>
+      </c>
+      <c r="V9" s="11"/>
+    </row>
+    <row r="10" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A10" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="55">
+        <f>_xlfn.BITAND($B$3,$B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="55">
+        <f>_xlfn.BITAND($D$3,$D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="55">
+        <f>_xlfn.BITAND($F$3,$F$4)</f>
+        <v>6</v>
+      </c>
+      <c r="G10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="55">
+        <f>_xlfn.BITAND($H$3,$H$4)+1</f>
+        <v>1</v>
+      </c>
+      <c r="I10" s="63"/>
+      <c r="J10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="55" t="str">
+        <f>DEC2BIN(B10,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" s="55" t="str">
+        <f>DEC2BIN(D10,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O10" s="55" t="str">
+        <f>DEC2BIN(F10,8)</f>
+        <v>00000110</v>
+      </c>
+      <c r="P10" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q10" s="55" t="str">
+        <f>DEC2BIN(H10,8)</f>
+        <v>00000001</v>
+      </c>
+      <c r="S10" s="11"/>
+      <c r="T10" s="16">
+        <v>255</v>
+      </c>
+      <c r="U10" s="11" t="str">
+        <f>DEC2BIN(T10,8)</f>
+        <v>11111111</v>
+      </c>
+      <c r="V10" s="11"/>
+    </row>
+    <row r="11" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A11" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" s="55">
+        <f>_xlfn.BITAND($B$3,$B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="55">
+        <f>_xlfn.BITAND($D$3,$D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="55">
+        <f>_xlfn.BITAND($F$3,$F$4)</f>
+        <v>6</v>
+      </c>
+      <c r="G11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="55">
+        <f>_xlfn.BITAND($H$3,$H$4)+2</f>
+        <v>2</v>
+      </c>
+      <c r="I11" s="63"/>
+      <c r="J11" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K11" s="55" t="str">
+        <f>DEC2BIN(B11,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M11" s="55" t="str">
+        <f>DEC2BIN(D11,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O11" s="55" t="str">
+        <f>DEC2BIN(F11,8)</f>
+        <v>00000110</v>
+      </c>
+      <c r="P11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q11" s="55" t="str">
+        <f>DEC2BIN(H11,8)</f>
+        <v>00000010</v>
+      </c>
+      <c r="T11" s="11">
+        <v>254</v>
+      </c>
+      <c r="U11" s="11" t="str">
+        <f>DEC2BIN(T11,8)</f>
+        <v>11111110</v>
+      </c>
+      <c r="V11" s="11"/>
+    </row>
+    <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A12" s="63"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="64"/>
+      <c r="H12" s="64"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="63"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="64"/>
+      <c r="M12" s="64"/>
+      <c r="N12" s="64"/>
+      <c r="O12" s="64"/>
+      <c r="P12" s="64"/>
+      <c r="Q12" s="64"/>
+      <c r="S12" s="11"/>
+      <c r="T12" s="16">
+        <v>252</v>
+      </c>
+      <c r="U12" s="11" t="str">
+        <f>DEC2BIN(T12,8)</f>
+        <v>11111100</v>
+      </c>
+      <c r="V12" s="11"/>
+    </row>
+    <row r="13" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A13" s="63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="64"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="64"/>
+      <c r="H13" s="64"/>
+      <c r="I13" s="63"/>
+      <c r="J13" s="63"/>
+      <c r="K13" s="64"/>
+      <c r="L13" s="64"/>
+      <c r="M13" s="64"/>
+      <c r="N13" s="64"/>
+      <c r="O13" s="64"/>
+      <c r="P13" s="64"/>
+      <c r="Q13" s="64"/>
+      <c r="T13" s="11">
+        <v>248</v>
+      </c>
+      <c r="U13" s="11" t="str">
+        <f>DEC2BIN(T13,8)</f>
+        <v>11111000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A14" s="63"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="63"/>
+      <c r="J14" s="63"/>
+      <c r="K14" s="64"/>
+      <c r="L14" s="64"/>
+      <c r="M14" s="64"/>
+      <c r="N14" s="64"/>
+      <c r="O14" s="64"/>
+      <c r="P14" s="64"/>
+      <c r="Q14" s="64"/>
+      <c r="T14" s="11">
+        <v>240</v>
+      </c>
+      <c r="U14" s="11" t="str">
+        <f>DEC2BIN(T14,8)</f>
+        <v>11110000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A15" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="55">
+        <f>_xlfn.BITAND($B$3,$B$4)+(255-$B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="55">
+        <f>_xlfn.BITAND($D$3,$D$4)+(255-$D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="55">
+        <f>_xlfn.BITAND($F$3,$F$4)+(255-$F$4)</f>
+        <v>7</v>
+      </c>
+      <c r="G15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="55">
+        <f>_xlfn.BITAND($H$3,$H$4)+(255-$H$4)-2</f>
+        <v>253</v>
+      </c>
+      <c r="I15" s="63"/>
+      <c r="J15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="55" t="str">
+        <f>DEC2BIN(B15,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="55" t="str">
+        <f>DEC2BIN(D15,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O15" s="55" t="str">
+        <f>DEC2BIN(F15,8)</f>
+        <v>00000111</v>
+      </c>
+      <c r="P15" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q15" s="55" t="str">
+        <f>DEC2BIN(H15,8)</f>
+        <v>11111101</v>
+      </c>
+      <c r="T15" s="11">
+        <v>224</v>
+      </c>
+      <c r="U15" s="11" t="str">
+        <f>DEC2BIN(T15,8)</f>
+        <v>11100000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A16" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="55">
+        <f>_xlfn.BITAND($B$3,$B$4)+(255-$B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="55">
+        <f>_xlfn.BITAND($D$3,$D$4)+(255-$D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="55">
+        <f>_xlfn.BITAND($F$3,$F$4)+(255-$F$4)</f>
+        <v>7</v>
+      </c>
+      <c r="G16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="55">
+        <f>_xlfn.BITAND($H$3,$H$4)+(255-$H$4)-1</f>
+        <v>254</v>
+      </c>
+      <c r="I16" s="63"/>
+      <c r="J16" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="55" t="str">
+        <f>DEC2BIN(B16,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M16" s="55" t="str">
+        <f>DEC2BIN(D16,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O16" s="55" t="str">
+        <f>DEC2BIN(F16,8)</f>
+        <v>00000111</v>
+      </c>
+      <c r="P16" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q16" s="55" t="str">
+        <f>DEC2BIN(H16,8)</f>
+        <v>11111110</v>
+      </c>
+      <c r="T16" s="11">
+        <v>192</v>
+      </c>
+      <c r="U16" s="11" t="str">
+        <f>DEC2BIN(T16,8)</f>
+        <v>11000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A17" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="62">
+        <f>_xlfn.BITAND($B$3,$B$4)+(255-$B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="62">
+        <f>_xlfn.BITAND($D$3,$D$4)+(255-$D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="62">
+        <f>_xlfn.BITAND($F$3,$F$4)+(255-$F$4)</f>
+        <v>7</v>
+      </c>
+      <c r="G17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="62">
+        <f>_xlfn.BITAND($H$3,$H$4)+(255-$H$4)</f>
+        <v>255</v>
+      </c>
+      <c r="I17" s="4"/>
+      <c r="J17" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="62" t="str">
+        <f>DEC2BIN(B17,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="M17" s="62" t="str">
+        <f>DEC2BIN(D17,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="O17" s="62" t="str">
+        <f>DEC2BIN(F17,8)</f>
+        <v>00000111</v>
+      </c>
+      <c r="P17" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q17" s="62" t="str">
+        <f>DEC2BIN(H17,8)</f>
+        <v>11111111</v>
+      </c>
+      <c r="T17" s="11">
+        <v>128</v>
+      </c>
+      <c r="U17" s="11" t="str">
+        <f>DEC2BIN(T17,8)</f>
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="T18" s="11">
+        <v>0</v>
+      </c>
+      <c r="U18" s="11" t="str">
+        <f>DEC2BIN(T18,8)</f>
+        <v>00000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A20" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="54"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="54"/>
+      <c r="L20" s="54"/>
+      <c r="M20" s="54"/>
+      <c r="N20" s="54"/>
+      <c r="O20" s="54"/>
+      <c r="P20" s="54"/>
+      <c r="Q20" s="54"/>
+    </row>
+    <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="55">
+        <v>192</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="55">
+        <v>168</v>
+      </c>
+      <c r="E21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" s="55">
+        <v>6</v>
+      </c>
+      <c r="G21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H21" s="55">
+        <v>13</v>
+      </c>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K21" s="55" t="str">
+        <f t="shared" ref="K21:K30" si="1">DEC2BIN(B21,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M21" s="55" t="str">
+        <f t="shared" ref="M21:M30" si="2">DEC2BIN(D21,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O21" s="55" t="str">
+        <f t="shared" ref="O21:O30" si="3">DEC2BIN(F21,8)</f>
+        <v>00000110</v>
+      </c>
+      <c r="P21" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q21" s="55" t="str">
+        <f t="shared" ref="Q21:Q30" si="4">DEC2BIN(H21,8)</f>
+        <v>00001101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A22" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="57">
+        <f>_xlfn.BITAND(B21,B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C22" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="57">
+        <f>_xlfn.BITAND(D21,D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E22" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="57">
+        <f>_xlfn.BITAND(F21,F$4)</f>
+        <v>6</v>
+      </c>
+      <c r="G22" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="H22" s="57">
+        <f>_xlfn.BITAND(H21,H$4)</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="54" t="str">
         <f t="shared" si="1"/>
         <v>11000000</v>
       </c>
-      <c r="L9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M9" s="12" t="str">
+      <c r="L22" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="M22" s="54" t="str">
         <f t="shared" si="2"/>
         <v>10101000</v>
       </c>
-      <c r="N9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O9" s="12" t="str">
+      <c r="N22" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="O22" s="54" t="str">
         <f t="shared" si="3"/>
-        <v>00000010</v>
-      </c>
-      <c r="P9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q9" s="12" t="str">
+        <v>00000110</v>
+      </c>
+      <c r="P22" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q22" s="54" t="str">
+        <f t="shared" si="4"/>
+        <v>00000000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A23" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="55">
+        <v>192</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="55">
+        <v>168</v>
+      </c>
+      <c r="E23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="55">
+        <v>7</v>
+      </c>
+      <c r="G23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="55">
+        <v>41</v>
+      </c>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K23" s="55" t="str">
+        <f t="shared" si="1"/>
+        <v>11000000</v>
+      </c>
+      <c r="L23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M23" s="55" t="str">
+        <f t="shared" si="2"/>
+        <v>10101000</v>
+      </c>
+      <c r="N23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="O23" s="55" t="str">
+        <f t="shared" si="3"/>
+        <v>00000111</v>
+      </c>
+      <c r="P23" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q23" s="55" t="str">
+        <f t="shared" si="4"/>
+        <v>00101001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A24" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="57">
+        <f>_xlfn.BITAND(B23,B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C24" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="57">
+        <f>_xlfn.BITAND(D23,D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E24" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="57">
+        <f>_xlfn.BITAND(F23,F$4)</f>
+        <v>6</v>
+      </c>
+      <c r="G24" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="H24" s="57">
+        <f>_xlfn.BITAND(H23,H$4)</f>
+        <v>0</v>
+      </c>
+      <c r="I24"/>
+      <c r="J24"/>
+      <c r="K24" s="54" t="str">
+        <f t="shared" si="1"/>
+        <v>11000000</v>
+      </c>
+      <c r="L24" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="M24" s="54" t="str">
+        <f t="shared" si="2"/>
+        <v>10101000</v>
+      </c>
+      <c r="N24" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="O24" s="54" t="str">
+        <f t="shared" si="3"/>
+        <v>00000110</v>
+      </c>
+      <c r="P24" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q24" s="54" t="str">
+        <f t="shared" si="4"/>
+        <v>00000000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A25" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="59">
+        <v>192</v>
+      </c>
+      <c r="C25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="59">
+        <v>168</v>
+      </c>
+      <c r="E25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25" s="59">
+        <v>8</v>
+      </c>
+      <c r="G25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25" s="59">
+        <v>255</v>
+      </c>
+      <c r="I25" s="58"/>
+      <c r="J25" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="K25" s="59" t="str">
+        <f>DEC2BIN(B25,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="M25" s="59" t="str">
+        <f>DEC2BIN(D25,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="O25" s="59" t="str">
+        <f>DEC2BIN(F25,8)</f>
+        <v>00001000</v>
+      </c>
+      <c r="P25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q25" s="59" t="str">
+        <f>DEC2BIN(H25,8)</f>
+        <v>11111111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A26" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26" s="57">
+        <f>_xlfn.BITAND(B25,B$4)</f>
+        <v>192</v>
+      </c>
+      <c r="C26" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="57">
+        <f>_xlfn.BITAND(D25,D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E26" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="57">
+        <f>_xlfn.BITAND(F25,F$4)</f>
+        <v>8</v>
+      </c>
+      <c r="G26" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26" s="57">
+        <f>_xlfn.BITAND(H25,H$4)</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="54" t="str">
+        <f>DEC2BIN(B26,8)</f>
+        <v>11000000</v>
+      </c>
+      <c r="L26" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="M26" s="54" t="str">
+        <f>DEC2BIN(D26,8)</f>
+        <v>10101000</v>
+      </c>
+      <c r="N26" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="O26" s="54" t="str">
+        <f>DEC2BIN(F26,8)</f>
+        <v>00001000</v>
+      </c>
+      <c r="P26" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q26" s="54" t="str">
+        <f>DEC2BIN(H26,8)</f>
+        <v>00000000</v>
+      </c>
+      <c r="V26" s="11"/>
+      <c r="W26" s="11"/>
+    </row>
+    <row r="27" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A27" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="59">
+        <v>10</v>
+      </c>
+      <c r="C27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" s="59">
+        <v>168</v>
+      </c>
+      <c r="E27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="F27" s="59">
+        <v>1</v>
+      </c>
+      <c r="G27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="H27" s="59">
+        <v>51</v>
+      </c>
+      <c r="I27" s="58"/>
+      <c r="J27" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="K27" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>00001010</v>
+      </c>
+      <c r="L27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="M27" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>10101000</v>
+      </c>
+      <c r="N27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="O27" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>00000001</v>
+      </c>
+      <c r="P27" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q27" s="59" t="str">
+        <f t="shared" si="4"/>
+        <v>00110011</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" ht="15" x14ac:dyDescent="0.4">
+      <c r="A28" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="57">
+        <f>_xlfn.BITAND(B27,B$4)</f>
+        <v>10</v>
+      </c>
+      <c r="C28" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="57">
+        <f>_xlfn.BITAND(D27,D$4)</f>
+        <v>168</v>
+      </c>
+      <c r="E28" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" s="57">
+        <f>_xlfn.BITAND(F27,F$4)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28" s="57">
+        <f>_xlfn.BITAND(H27,H$4)</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11" t="str">
+        <f t="shared" si="1"/>
+        <v>00001010</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M28" s="11" t="str">
+        <f t="shared" si="2"/>
+        <v>10101000</v>
+      </c>
+      <c r="N28" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="O28" s="11" t="str">
+        <f t="shared" si="3"/>
+        <v>00000000</v>
+      </c>
+      <c r="P28" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q28" s="11" t="str">
+        <f t="shared" si="4"/>
+        <v>00000000</v>
+      </c>
+      <c r="V28" s="11"/>
+      <c r="W28" s="11"/>
+    </row>
+    <row r="29" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A29" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="59">
+        <v>192</v>
+      </c>
+      <c r="C29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="59">
+        <v>168</v>
+      </c>
+      <c r="E29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="59">
+        <v>50</v>
+      </c>
+      <c r="G29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="H29" s="59">
+        <v>23</v>
+      </c>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="K29" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>11000000</v>
+      </c>
+      <c r="L29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="M29" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>10101000</v>
+      </c>
+      <c r="N29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="O29" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>00110010</v>
+      </c>
+      <c r="P29" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q29" s="59" t="str">
         <f t="shared" si="4"/>
         <v>00010111</v>
       </c>
-      <c r="S9" s="11">
+    </row>
+    <row r="30" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A30" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="57">
+        <f>_xlfn.BITAND(B29,B$4)</f>
         <v>192</v>
       </c>
-      <c r="T9" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>11000000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A10" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="12">
-        <v>192</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="12">
+      <c r="C30" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="57">
+        <f>_xlfn.BITAND(D29,D$4)</f>
         <v>168</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="12">
-        <v>2</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" s="12">
-        <v>233</v>
-      </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K10" s="12" t="str">
+      <c r="E30" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="57">
+        <f>_xlfn.BITAND(F29,F$4)</f>
+        <v>50</v>
+      </c>
+      <c r="G30" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="H30" s="57">
+        <f>_xlfn.BITAND(H29,H$4)</f>
+        <v>0</v>
+      </c>
+      <c r="I30"/>
+      <c r="J30"/>
+      <c r="K30" s="54" t="str">
         <f t="shared" si="1"/>
         <v>11000000</v>
       </c>
-      <c r="L10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M10" s="12" t="str">
+      <c r="L30" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="M30" s="54" t="str">
         <f t="shared" si="2"/>
         <v>10101000</v>
       </c>
-      <c r="N10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O10" s="12" t="str">
+      <c r="N30" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="O30" s="54" t="str">
         <f t="shared" si="3"/>
-        <v>00000010</v>
-      </c>
-      <c r="P10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q10" s="12" t="str">
+        <v>00110010</v>
+      </c>
+      <c r="P30" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q30" s="54" t="str">
         <f t="shared" si="4"/>
-        <v>11101001</v>
-      </c>
-      <c r="S10" s="11">
-        <v>128</v>
-      </c>
-      <c r="T10" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A11" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="12">
-        <v>192</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="12">
-        <v>168</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="12">
-        <v>2</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" s="12">
-        <v>6</v>
-      </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K11" s="12" t="str">
-        <f>DEC2BIN(B11,8)</f>
-        <v>11000000</v>
-      </c>
-      <c r="L11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M11" s="12" t="str">
-        <f>DEC2BIN(D11,8)</f>
-        <v>10101000</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O11" s="12" t="str">
-        <f>DEC2BIN(F11,8)</f>
-        <v>00000010</v>
-      </c>
-      <c r="P11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q11" s="12" t="str">
-        <f>DEC2BIN(H11,8)</f>
-        <v>00000110</v>
-      </c>
-      <c r="S11" s="11">
-        <v>0</v>
-      </c>
-      <c r="T11" s="11" t="str">
-        <f t="shared" si="0"/>
         <v>00000000</v>
       </c>
-    </row>
-    <row r="12" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A12" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="13">
-        <v>255</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="13">
-        <v>255</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="13">
-        <v>255</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="13">
-        <v>0</v>
-      </c>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K12" s="13" t="str">
-        <f>DEC2BIN(B12,8)</f>
-        <v>11111111</v>
-      </c>
-      <c r="L12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="M12" s="13" t="str">
-        <f>DEC2BIN(D12,8)</f>
-        <v>11111111</v>
-      </c>
-      <c r="N12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="O12" s="13" t="str">
-        <f>DEC2BIN(F12,8)</f>
-        <v>11111111</v>
-      </c>
-      <c r="P12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q12" s="13" t="str">
-        <f>DEC2BIN(H12,8)</f>
-        <v>00000000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="T13" s="11"/>
-    </row>
-    <row r="14" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A14" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="15">
-        <f>_xlfn.BITAND(B11,B12)</f>
-        <v>192</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="15">
-        <f t="shared" ref="D14:H14" si="5">_xlfn.BITAND(D11,D12)</f>
-        <v>168</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="15">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" s="15">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="K14" s="15" t="str">
-        <f>DEC2BIN(B14,8)</f>
-        <v>11000000</v>
-      </c>
-      <c r="L14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="M14" s="15" t="str">
-        <f t="shared" ref="M14:Q14" si="6">DEC2BIN(D14,8)</f>
-        <v>10101000</v>
-      </c>
-      <c r="N14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O14" s="15" t="str">
-        <f t="shared" si="6"/>
-        <v>00000010</v>
-      </c>
-      <c r="P14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q14" s="15" t="str">
-        <f t="shared" si="6"/>
-        <v>00000000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-    </row>
-    <row r="16" spans="1:20" ht="15" x14ac:dyDescent="0.4">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
+      <c r="S30"/>
+      <c r="T30"/>
+      <c r="U30"/>
+    </row>
+    <row r="31" spans="1:23" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+      <c r="A31"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="54"/>
+      <c r="M31" s="54"/>
+      <c r="N31" s="54"/>
+      <c r="O31" s="54"/>
+      <c r="P31" s="54"/>
+      <c r="Q31" s="54"/>
+      <c r="U31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3684,7 +5426,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763721F9-D241-4071-831B-604643AF0551}">
-  <dimension ref="A1:W47"/>
+  <dimension ref="A1:W36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.1796875" customWidth="1"/>
@@ -3703,735 +5445,518 @@
   <sheetData>
     <row r="1" spans="1:23" ht="31" x14ac:dyDescent="0.7">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
+        <v>61</v>
+      </c>
       <c r="I3" s="20"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
       <c r="R3" s="20"/>
       <c r="S3" s="20"/>
       <c r="T3" s="20"/>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-    </row>
     <row r="5" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1"/>
-      <c r="I5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
     </row>
     <row r="6" spans="1:23" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="1"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="45" t="s">
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+      <c r="M7" s="49"/>
+      <c r="N7" s="49"/>
+      <c r="O7" s="49"/>
+      <c r="P7" s="50"/>
+      <c r="Q7" s="35"/>
+      <c r="R7" s="48" t="s">
+        <v>71</v>
+      </c>
+      <c r="S7" s="49"/>
+      <c r="T7" s="49"/>
+      <c r="U7" s="50"/>
+      <c r="V7" s="35"/>
+      <c r="W7" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="46"/>
-      <c r="L7" s="46"/>
-      <c r="M7" s="46"/>
-      <c r="N7" s="46"/>
-      <c r="O7" s="46"/>
-      <c r="P7" s="47"/>
-      <c r="Q7" s="48"/>
-      <c r="R7" s="45" t="s">
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A8" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="28">
+        <v>192</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="27">
+        <v>168</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="27">
+        <v>1</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="29">
+        <v>1</v>
+      </c>
+      <c r="I8" s="27"/>
+      <c r="J8" s="28">
+        <v>255</v>
+      </c>
+      <c r="K8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="27">
+        <v>255</v>
+      </c>
+      <c r="M8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="N8" s="27">
+        <v>255</v>
+      </c>
+      <c r="O8" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="P8" s="29">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="27"/>
+      <c r="R8" s="28"/>
+      <c r="S8" s="27"/>
+      <c r="T8" s="27"/>
+      <c r="U8" s="29"/>
+      <c r="W8" s="33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A9" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="31">
+        <v>192</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="30">
+        <v>168</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="30">
+        <v>2</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="32">
+        <v>1</v>
+      </c>
+      <c r="I9" s="30"/>
+      <c r="J9" s="31">
+        <v>255</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="30">
+        <v>255</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="N9" s="30">
+        <v>255</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="P9" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="31"/>
+      <c r="S9" s="30"/>
+      <c r="T9" s="30"/>
+      <c r="U9" s="32"/>
+      <c r="W9" s="33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A10" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="51" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="52"/>
+      <c r="D10" s="52"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="52"/>
+      <c r="J10" s="52"/>
+      <c r="K10" s="52"/>
+      <c r="L10" s="52"/>
+      <c r="M10" s="52"/>
+      <c r="N10" s="52"/>
+      <c r="O10" s="52"/>
+      <c r="P10" s="52"/>
+      <c r="Q10" s="52"/>
+      <c r="R10" s="52"/>
+      <c r="S10" s="52"/>
+      <c r="T10" s="52"/>
+      <c r="U10" s="53"/>
+      <c r="W10" s="33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B11" s="22"/>
+      <c r="H11" s="23"/>
+      <c r="J11" s="22"/>
+      <c r="P11" s="23"/>
+      <c r="R11" s="22"/>
+      <c r="U11" s="23"/>
+      <c r="W11" s="33"/>
+    </row>
+    <row r="12" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="25"/>
+      <c r="N12" s="25"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="26"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="25"/>
+      <c r="T12" s="25"/>
+      <c r="U12" s="26"/>
+      <c r="W12" s="34"/>
+    </row>
+    <row r="14" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+    </row>
+    <row r="16" spans="1:23" ht="17" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A17" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="45">
+        <v>192</v>
+      </c>
+      <c r="C17" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="45">
+        <v>168</v>
+      </c>
+      <c r="E17" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="45">
+        <v>2</v>
+      </c>
+      <c r="G17" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="46">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A22" s="41"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="41"/>
+      <c r="L22" s="41"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A23" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="S7" s="46"/>
-      <c r="T7" s="46"/>
-      <c r="U7" s="47"/>
-      <c r="V7" s="48"/>
-      <c r="W7" s="53" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A8" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" s="33">
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="41"/>
+      <c r="L23" s="41"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A24" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="41"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="41"/>
+      <c r="K24" s="41"/>
+      <c r="L24" s="41"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="41"/>
+      <c r="C25" s="41"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="41"/>
+      <c r="K25" s="41"/>
+      <c r="L25" s="41"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A26" s="41"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41"/>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="41"/>
+      <c r="K26" s="41"/>
+      <c r="L26" s="41"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="41"/>
+      <c r="I27" s="41"/>
+      <c r="J27" s="41"/>
+      <c r="K27" s="41"/>
+      <c r="L27" s="41"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A28" s="41"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="41"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="41"/>
+      <c r="K28" s="41"/>
+      <c r="L28" s="41"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A29" s="41"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="47" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="47"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="44" t="s">
+        <v>80</v>
+      </c>
+      <c r="I29" s="41"/>
+      <c r="J29" s="41"/>
+      <c r="K29" s="41"/>
+      <c r="L29" s="41"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A30" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" s="41"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="42">
+        <v>3</v>
+      </c>
+      <c r="G30" s="41"/>
+      <c r="H30" s="43" t="str">
+        <f>IF(F30=1,"👈  eins", "👈 nicht eins")</f>
+        <v>👈 nicht eins</v>
+      </c>
+      <c r="I30" s="41"/>
+      <c r="J30" s="41"/>
+      <c r="K30" s="41"/>
+      <c r="L30" s="41"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A31" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="41"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="41"/>
+      <c r="F31" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="G31" s="41"/>
+      <c r="H31" s="43" t="str">
+        <f>F31</f>
+        <v>Hallo</v>
+      </c>
+      <c r="I31" s="41"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A32" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="42">
+        <v>255</v>
+      </c>
+      <c r="E32" s="41"/>
+      <c r="F32" s="42">
         <v>192</v>
       </c>
-      <c r="C8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="34">
-        <v>168</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="34">
-        <v>1</v>
-      </c>
-      <c r="G8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="35">
-        <v>1</v>
-      </c>
-      <c r="I8" s="32"/>
-      <c r="J8" s="33">
-        <v>255</v>
-      </c>
-      <c r="K8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" s="34">
-        <v>255</v>
-      </c>
-      <c r="M8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="N8" s="34">
-        <v>255</v>
-      </c>
-      <c r="O8" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="P8" s="35">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="32"/>
-      <c r="R8" s="33"/>
-      <c r="S8" s="34"/>
-      <c r="T8" s="34"/>
-      <c r="U8" s="35"/>
-      <c r="W8" s="43" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A9" s="50" t="s">
-        <v>67</v>
-      </c>
-      <c r="B9" s="37">
+      <c r="G32" s="41"/>
+      <c r="H32" s="43">
+        <f>_xlfn.BITAND(F32,D32)</f>
         <v>192</v>
       </c>
-      <c r="C9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="38">
-        <v>168</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="38">
-        <v>2</v>
-      </c>
-      <c r="G9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="39">
-        <v>1</v>
-      </c>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37">
-        <v>255</v>
-      </c>
-      <c r="K9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="L9" s="38">
-        <v>255</v>
-      </c>
-      <c r="M9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="N9" s="38">
-        <v>255</v>
-      </c>
-      <c r="O9" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="P9" s="39">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="36"/>
-      <c r="R9" s="37"/>
-      <c r="S9" s="38"/>
-      <c r="T9" s="38"/>
-      <c r="U9" s="39"/>
-      <c r="W9" s="43" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A10" s="51" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="41"/>
-      <c r="R10" s="41"/>
-      <c r="S10" s="41"/>
-      <c r="T10" s="41"/>
-      <c r="U10" s="42"/>
-      <c r="W10" s="43" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="26"/>
-      <c r="P11" s="27"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="26"/>
-      <c r="T11" s="26"/>
-      <c r="U11" s="27"/>
-      <c r="W11" s="43"/>
-    </row>
-    <row r="12" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="31"/>
-      <c r="J12" s="29"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="31"/>
-      <c r="R12" s="29"/>
-      <c r="S12" s="30"/>
-      <c r="T12" s="30"/>
-      <c r="U12" s="31"/>
-      <c r="W12" s="44"/>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="21"/>
-      <c r="O13" s="21"/>
-      <c r="P13" s="21"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="21"/>
-    </row>
-    <row r="14" spans="1:23" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="21"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21"/>
-      <c r="L14" s="21"/>
-      <c r="M14" s="21"/>
-      <c r="N14" s="21"/>
-      <c r="O14" s="21"/>
-      <c r="P14" s="21"/>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="21"/>
-    </row>
-    <row r="15" spans="1:23" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="21"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="21"/>
-      <c r="P15" s="21"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
-    </row>
-    <row r="16" spans="1:23" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="21"/>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
-      <c r="P17" s="21"/>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="21"/>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="J18" s="21"/>
-    </row>
-    <row r="25" spans="1:22" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="21"/>
-      <c r="O25" s="21"/>
-      <c r="P25" s="21"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="21"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="21"/>
-      <c r="O26" s="21"/>
-      <c r="P26" s="21"/>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="21"/>
-    </row>
-    <row r="27" spans="1:22" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A27" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="J27" s="28"/>
-      <c r="K27" s="28"/>
-      <c r="L27" s="28"/>
-      <c r="M27" s="28"/>
-      <c r="N27" s="28"/>
-      <c r="O27" s="28"/>
-      <c r="P27" s="28"/>
-      <c r="Q27" s="28"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
-      <c r="V27" s="28"/>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="J28" s="52"/>
-      <c r="K28" s="52"/>
-      <c r="L28" s="52"/>
-      <c r="M28" s="52"/>
-      <c r="N28" s="52"/>
-      <c r="O28" s="52"/>
-      <c r="P28" s="52"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="52"/>
-      <c r="S28" s="52"/>
-      <c r="T28" s="52"/>
-      <c r="U28" s="52"/>
-      <c r="V28" s="28"/>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A29" s="54" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" s="60">
-        <v>192</v>
-      </c>
-      <c r="C29" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29" s="60">
-        <v>168</v>
-      </c>
-      <c r="E29" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="F29" s="60">
-        <v>2</v>
-      </c>
-      <c r="G29" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="H29" s="61">
-        <v>12</v>
-      </c>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
-      <c r="V29" s="28"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="21"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="28"/>
-      <c r="L30" s="28"/>
-      <c r="M30" s="28"/>
-      <c r="N30" s="28"/>
-      <c r="O30" s="28"/>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
-      <c r="V30" s="28"/>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
-      <c r="M31" s="28"/>
-      <c r="N31" s="28"/>
-      <c r="O31" s="28"/>
-      <c r="P31" s="28"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
-      <c r="V31" s="28"/>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="41"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A33" s="55"/>
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="55"/>
-      <c r="J33" s="55"/>
-      <c r="K33" s="55"/>
-      <c r="L33" s="55"/>
+      <c r="A33" s="41"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A34" s="55" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" s="55"/>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55"/>
-      <c r="L34" s="55"/>
+      <c r="A34" s="41"/>
+      <c r="B34" s="41"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="42"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="42"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="41"/>
+      <c r="K34" s="41"/>
+      <c r="L34" s="41"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A35" s="55" t="s">
-        <v>74</v>
-      </c>
-      <c r="B35" s="55"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="55"/>
-      <c r="J35" s="55"/>
-      <c r="K35" s="55"/>
-      <c r="L35" s="55"/>
+      <c r="A35" s="41"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="41"/>
+      <c r="K35" s="41"/>
+      <c r="L35" s="41"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A36" s="55" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="55"/>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
-      <c r="J36" s="55"/>
-      <c r="K36" s="55"/>
-      <c r="L36" s="55"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A37" s="55"/>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
-      <c r="I37" s="55"/>
-      <c r="J37" s="55"/>
-      <c r="K37" s="55"/>
-      <c r="L37" s="55"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A38" s="55" t="s">
-        <v>76</v>
-      </c>
-      <c r="B38" s="55"/>
-      <c r="C38" s="55"/>
-      <c r="D38" s="55"/>
-      <c r="E38" s="55"/>
-      <c r="F38" s="55"/>
-      <c r="G38" s="55"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="55"/>
-      <c r="K38" s="55"/>
-      <c r="L38" s="55"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A39" s="55"/>
-      <c r="B39" s="55"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
-      <c r="I39" s="55"/>
-      <c r="J39" s="55"/>
-      <c r="K39" s="55"/>
-      <c r="L39" s="55"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A40" s="55"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="59" t="s">
-        <v>80</v>
-      </c>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="58" t="s">
-        <v>81</v>
-      </c>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
-      <c r="K40" s="55"/>
-      <c r="L40" s="55"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A41" s="55" t="s">
-        <v>75</v>
-      </c>
-      <c r="B41" s="55"/>
-      <c r="C41" s="55"/>
-      <c r="D41" s="56"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="56">
-        <v>3</v>
-      </c>
-      <c r="G41" s="55"/>
-      <c r="H41" s="57" t="str">
-        <f>IF(F41=1,"👈  eins", "👈 nicht eins")</f>
-        <v>👈 nicht eins</v>
-      </c>
-      <c r="I41" s="55"/>
-      <c r="J41" s="55"/>
-      <c r="K41" s="55"/>
-      <c r="L41" s="55"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A42" s="55" t="s">
-        <v>78</v>
-      </c>
-      <c r="B42" s="55"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="56"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="56" t="s">
-        <v>79</v>
-      </c>
-      <c r="G42" s="55"/>
-      <c r="H42" s="57" t="str">
-        <f>F42</f>
-        <v>Hallo</v>
-      </c>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55"/>
-      <c r="K42" s="55"/>
-      <c r="L42" s="55"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A43" s="55" t="s">
-        <v>82</v>
-      </c>
-      <c r="B43" s="55"/>
-      <c r="C43" s="55"/>
-      <c r="D43" s="56">
-        <v>255</v>
-      </c>
-      <c r="E43" s="55"/>
-      <c r="F43" s="56">
-        <v>192</v>
-      </c>
-      <c r="G43" s="55"/>
-      <c r="H43" s="57">
-        <f>_xlfn.BITAND(F43,D43)</f>
-        <v>192</v>
-      </c>
-      <c r="I43" s="55"/>
-      <c r="J43" s="55"/>
-      <c r="K43" s="55"/>
-      <c r="L43" s="55"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A44" s="55"/>
-      <c r="B44" s="55"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="56"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="55"/>
-      <c r="H44" s="57"/>
-      <c r="I44" s="55"/>
-      <c r="J44" s="55"/>
-      <c r="K44" s="55"/>
-      <c r="L44" s="55"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A45" s="55"/>
-      <c r="B45" s="55"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="55"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="55"/>
-      <c r="H45" s="57"/>
-      <c r="I45" s="55"/>
-      <c r="J45" s="55"/>
-      <c r="K45" s="55"/>
-      <c r="L45" s="55"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A46" s="55"/>
-      <c r="B46" s="55"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="55"/>
-      <c r="H46" s="55"/>
-      <c r="I46" s="55"/>
-      <c r="J46" s="55"/>
-      <c r="K46" s="55"/>
-      <c r="L46" s="55"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A47" s="55"/>
-      <c r="B47" s="55"/>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="55"/>
-      <c r="F47" s="55"/>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="55"/>
-      <c r="J47" s="55"/>
-      <c r="K47" s="55"/>
-      <c r="L47" s="55"/>
+      <c r="A36" s="41"/>
+      <c r="B36" s="41"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
+      <c r="H36" s="41"/>
+      <c r="I36" s="41"/>
+      <c r="J36" s="41"/>
+      <c r="K36" s="41"/>
+      <c r="L36" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="D29:F29"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="J7:P7"/>
     <mergeCell ref="R7:U7"/>

</xml_diff>